<commit_message>
Updated_Role 4: ablations, consolidated results, paper draft skeleton
</commit_message>
<xml_diff>
--- a/outputs/consolidated_results.xlsx
+++ b/outputs/consolidated_results.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,27 +447,57 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>accuracy</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>macro_f1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>precision</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>recall</t>
+          <t>nonhate_precision</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>nonhate_recall</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>nonhate_f1</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>hate_precision</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>hate_recall</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>hate_f1</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>macro_precision</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>macro_recall</t>
         </is>
       </c>
     </row>
@@ -483,19 +513,37 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9</v>
+        <v>5029</v>
       </c>
       <c r="D2" t="n">
-        <v>0.88</v>
+        <v>0.9270232650626368</v>
       </c>
       <c r="E2" t="n">
-        <v>0.91</v>
+        <v>0.9269254426052832</v>
       </c>
       <c r="F2" t="n">
-        <v>0.89</v>
+        <v>0.931923076923077</v>
       </c>
       <c r="G2" t="n">
-        <v>600</v>
+        <v>0.9272866437045542</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9295990792250144</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.9217785096747632</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.9267384105960264</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.924251805985552</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.92685079329892</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.9270125271502904</v>
       </c>
     </row>
     <row r="3">
@@ -510,19 +558,37 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.87</v>
+        <v>3060</v>
       </c>
       <c r="D3" t="n">
-        <v>0.85</v>
+        <v>0.842156862745098</v>
       </c>
       <c r="E3" t="n">
-        <v>0.88</v>
+        <v>0.8412988330796549</v>
       </c>
       <c r="F3" t="n">
-        <v>0.86</v>
+        <v>0.8060989643268124</v>
       </c>
       <c r="G3" t="n">
-        <v>600</v>
+        <v>0.9056237879767292</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8529680365296803</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.8895612708018155</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.7772637144745539</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.8296296296296296</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8478301175643139</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.8414437512256415</v>
       </c>
     </row>
     <row r="4">
@@ -537,19 +603,37 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.852</v>
+        <v>3061</v>
       </c>
       <c r="D4" t="n">
-        <v>0.832</v>
+        <v>0.9081999346618752</v>
       </c>
       <c r="E4" t="n">
-        <v>0.862</v>
+        <v>0.908198523796752</v>
       </c>
       <c r="F4" t="n">
-        <v>0.842</v>
+        <v>0.9154098360655738</v>
       </c>
       <c r="G4" t="n">
-        <v>600</v>
+        <v>0.9018087855297158</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.9085584119752684</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.9010416666666666</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.914738929279577</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.9078386356182356</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.9082257513661204</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.9082738574046464</v>
       </c>
     </row>
     <row r="5">
@@ -564,19 +648,37 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8340000000000001</v>
+        <v>3061</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8140000000000001</v>
+        <v>0.9160405096373734</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8440000000000001</v>
+        <v>0.9159990547882204</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8240000000000001</v>
+        <v>0.9082858950031626</v>
       </c>
       <c r="G5" t="n">
-        <v>600</v>
+        <v>0.9276485788113696</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.9178651326302332</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9243243243243244</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.9041639127561136</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.9141329769462078</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.9163051096637436</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.9159062457837416</v>
       </c>
     </row>
     <row r="6">
@@ -591,19 +693,37 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9</v>
+        <v>5029</v>
       </c>
       <c r="D6" t="n">
-        <v>0.88</v>
+        <v>0.905746669317956</v>
       </c>
       <c r="E6" t="n">
-        <v>0.91</v>
+        <v>0.9053610875106202</v>
       </c>
       <c r="F6" t="n">
-        <v>0.89</v>
+        <v>0.8907563025210085</v>
       </c>
       <c r="G6" t="n">
-        <v>600</v>
+        <v>0.933027171833142</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.9114018691588786</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9236474694589878</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.8762417218543046</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.8993203058623619</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.9072018859899982</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.9046344468437232</v>
       </c>
     </row>
     <row r="7">
@@ -618,19 +738,37 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.87</v>
+        <v>3060</v>
       </c>
       <c r="D7" t="n">
-        <v>0.85</v>
+        <v>0.822875816993464</v>
       </c>
       <c r="E7" t="n">
-        <v>0.88</v>
+        <v>0.8213586360128892</v>
       </c>
       <c r="F7" t="n">
-        <v>0.86</v>
+        <v>0.7799442896935933</v>
       </c>
       <c r="G7" t="n">
-        <v>600</v>
+        <v>0.9049773755656108</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.8378216636744464</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.8837944664031621</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.7389292795769994</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.8048956083513319</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.8318693780483777</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.8219533275713051</v>
       </c>
     </row>
     <row r="8">
@@ -645,19 +783,37 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.852</v>
+        <v>3061</v>
       </c>
       <c r="D8" t="n">
-        <v>0.832</v>
+        <v>0.8846782097353806</v>
       </c>
       <c r="E8" t="n">
-        <v>0.862</v>
+        <v>0.8845646682524073</v>
       </c>
       <c r="F8" t="n">
-        <v>0.842</v>
+        <v>0.8713486637663145</v>
       </c>
       <c r="G8" t="n">
-        <v>600</v>
+        <v>0.9056847545219638</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8881849857459614</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.8994490358126722</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.8631857237276933</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.8809443507588532</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.8853988497894933</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.8844352391248286</v>
       </c>
     </row>
     <row r="9">
@@ -672,19 +828,37 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8340000000000001</v>
+        <v>3061</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8140000000000001</v>
+        <v>0.8908853315909834</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8440000000000001</v>
+        <v>0.8906466728104605</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8240000000000001</v>
+        <v>0.8665458937198067</v>
       </c>
       <c r="G9" t="n">
-        <v>600</v>
+        <v>0.9270025839793282</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.8957553058676654</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9195729537366548</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.8539325842696629</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.8855380397532556</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.8930594237282308</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.8904675841244956</v>
       </c>
     </row>
   </sheetData>
@@ -698,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -760,19 +934,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.9</v>
+        <v>0.9270232650626368</v>
       </c>
       <c r="E2" t="n">
-        <v>0.04</v>
+        <v>0.0357962132354742</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1</v>
+        <v>0.2504876644999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08</v>
+        <v>0.0576771630429045</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3</v>
+        <v>0.2100434758228277</v>
       </c>
     </row>
     <row r="3">
@@ -783,28 +957,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.9</v>
+        <v>0.842156862745098</v>
       </c>
       <c r="E3" t="n">
-        <v>0.018</v>
+        <v>0.09196641473290849</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04500000000000001</v>
+        <v>0.2132337654673539</v>
       </c>
       <c r="G3" t="n">
-        <v>0.036</v>
+        <v>0.1284985317819034</v>
       </c>
       <c r="H3" t="n">
-        <v>0.135</v>
+        <v>0.4507268863367671</v>
       </c>
     </row>
     <row r="4">
@@ -815,28 +989,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.9</v>
+        <v>0.9081999346618752</v>
       </c>
       <c r="E4" t="n">
-        <v>0.016</v>
+        <v>0.0432784854988566</v>
       </c>
       <c r="F4" t="n">
-        <v>0.04000000000000001</v>
+        <v>0.2699211897727273</v>
       </c>
       <c r="G4" t="n">
-        <v>0.032</v>
+        <v>0.0714346859932366</v>
       </c>
       <c r="H4" t="n">
-        <v>0.12</v>
+        <v>0.2515337383255857</v>
       </c>
     </row>
     <row r="5">
@@ -847,7 +1021,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -856,57 +1030,57 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.87</v>
+        <v>0.9160405096373734</v>
       </c>
       <c r="E5" t="n">
-        <v>0.09</v>
+        <v>0.0456853069535773</v>
       </c>
       <c r="F5" t="n">
-        <v>0.18</v>
+        <v>0.3932348841463415</v>
       </c>
       <c r="G5" t="n">
-        <v>0.13</v>
+        <v>0.0672258913774315</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5</v>
+        <v>0.2517113006655102</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>banglabert</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_standard</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.87</v>
+        <v>0.905746669317956</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0405</v>
+        <v>0.0293490971321137</v>
       </c>
       <c r="F6" t="n">
-        <v>0.081</v>
+        <v>0.2352363794565218</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0585</v>
+        <v>0.072799843846375</v>
       </c>
       <c r="H6" t="n">
-        <v>0.225</v>
+        <v>0.2492301813170459</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>banglabert</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -916,29 +1090,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.87</v>
+        <v>0.822875816993464</v>
       </c>
       <c r="E7" t="n">
-        <v>0.036</v>
+        <v>0.0523946958365686</v>
       </c>
       <c r="F7" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.2071042125423728</v>
       </c>
       <c r="G7" t="n">
-        <v>0.052</v>
+        <v>0.1293861312762249</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2</v>
+        <v>0.4115922358487386</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>banglabert</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -952,51 +1126,51 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.852</v>
+        <v>0.8846782097353806</v>
       </c>
       <c r="E8" t="n">
-        <v>0.12</v>
+        <v>0.0208834329419144</v>
       </c>
       <c r="F8" t="n">
-        <v>0.228</v>
+        <v>0.1821227487878788</v>
       </c>
       <c r="G8" t="n">
-        <v>0.16</v>
+        <v>0.0868247207788462</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6200000000000001</v>
+        <v>0.2878737777607087</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>banglabert</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.852</v>
+        <v>0.8908853315909834</v>
       </c>
       <c r="E9" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.032242713501078</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1026</v>
+        <v>0.2021496351376147</v>
       </c>
       <c r="G9" t="n">
-        <v>0.07200000000000002</v>
+        <v>0.0819480070115565</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2790000000000001</v>
+        <v>0.2754970172988697</v>
       </c>
     </row>
     <row r="10">
@@ -1007,28 +1181,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_standard</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.852</v>
+        <v>0.9270232650626368</v>
       </c>
       <c r="E10" t="n">
-        <v>0.04800000000000001</v>
+        <v>0.0186194421097822</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0912</v>
+        <v>0.2398671395156342</v>
       </c>
       <c r="G10" t="n">
-        <v>0.06400000000000002</v>
+        <v>0.0559425852403206</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2480000000000001</v>
+        <v>0.1961626501038725</v>
       </c>
     </row>
     <row r="11">
@@ -1039,28 +1213,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>test_dialect_barishal</t>
+          <t>test_standard</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>dirichlet</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.9284151918870552</v>
       </c>
       <c r="E11" t="n">
-        <v>0.15</v>
+        <v>0.0132889426712944</v>
       </c>
       <c r="F11" t="n">
-        <v>0.276</v>
+        <v>0.1651999197358278</v>
       </c>
       <c r="G11" t="n">
-        <v>0.19</v>
+        <v>0.0554116859382257</v>
       </c>
       <c r="H11" t="n">
-        <v>0.74</v>
+        <v>0.1943654634569975</v>
       </c>
     </row>
     <row r="12">
@@ -1071,7 +1245,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>test_dialect_barishal</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1080,19 +1254,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.842156862745098</v>
       </c>
       <c r="E12" t="n">
-        <v>0.06750000000000002</v>
+        <v>0.0687064124433315</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1242</v>
+        <v>0.1822910585955848</v>
       </c>
       <c r="G12" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.123263785334435</v>
       </c>
       <c r="H12" t="n">
-        <v>0.333</v>
+        <v>0.4055934138377777</v>
       </c>
     </row>
     <row r="13">
@@ -1103,7 +1277,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>test_dialect_barishal</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1112,147 +1286,147 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.8431372549019608</v>
       </c>
       <c r="E13" t="n">
-        <v>0.06000000000000001</v>
+        <v>0.0535748669046049</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1104</v>
+        <v>0.1665499283296937</v>
       </c>
       <c r="G13" t="n">
-        <v>0.07600000000000001</v>
+        <v>0.1203585119148847</v>
       </c>
       <c r="H13" t="n">
-        <v>0.296</v>
+        <v>0.3884791769529926</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>xlmr_base</t>
+          <t>banglabert</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.9</v>
+        <v>0.9081999346618752</v>
       </c>
       <c r="E14" t="n">
-        <v>0.04</v>
+        <v>0.0239193824382681</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1</v>
+        <v>0.1990885356081815</v>
       </c>
       <c r="G14" t="n">
-        <v>0.08</v>
+        <v>0.069036490919951</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3</v>
+        <v>0.234456968444127</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>xlmr_base</t>
+          <t>banglabert</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>dirichlet</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.9</v>
+        <v>0.9091800065338124</v>
       </c>
       <c r="E15" t="n">
-        <v>0.018</v>
+        <v>0.0232057320439756</v>
       </c>
       <c r="F15" t="n">
-        <v>0.04500000000000001</v>
+        <v>0.2307953522297094</v>
       </c>
       <c r="G15" t="n">
-        <v>0.036</v>
+        <v>0.0685317260566574</v>
       </c>
       <c r="H15" t="n">
-        <v>0.135</v>
+        <v>0.2330708521009007</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>xlmr_base</t>
+          <t>banglabert</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.9</v>
+        <v>0.9160405096373734</v>
       </c>
       <c r="E16" t="n">
-        <v>0.016</v>
+        <v>0.0316692294786609</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04000000000000001</v>
+        <v>0.2556276976209362</v>
       </c>
       <c r="G16" t="n">
-        <v>0.032</v>
+        <v>0.0650309562919436</v>
       </c>
       <c r="H16" t="n">
-        <v>0.12</v>
+        <v>0.2292197963682935</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>xlmr_base</t>
+          <t>banglabert</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>dirichlet</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.87</v>
+        <v>0.9173472721332898</v>
       </c>
       <c r="E17" t="n">
-        <v>0.09</v>
+        <v>0.0228566995334894</v>
       </c>
       <c r="F17" t="n">
-        <v>0.18</v>
+        <v>0.3325478398398973</v>
       </c>
       <c r="G17" t="n">
-        <v>0.13</v>
+        <v>0.0639371717081839</v>
       </c>
       <c r="H17" t="n">
-        <v>0.5</v>
+        <v>0.2229379098677356</v>
       </c>
     </row>
     <row r="18">
@@ -1263,7 +1437,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_standard</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1272,19 +1446,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.87</v>
+        <v>0.905746669317956</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0405</v>
+        <v>0.0255101253562159</v>
       </c>
       <c r="F18" t="n">
-        <v>0.081</v>
+        <v>0.1774103995270195</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0585</v>
+        <v>0.0721349099995602</v>
       </c>
       <c r="H18" t="n">
-        <v>0.225</v>
+        <v>0.2452316843215874</v>
       </c>
     </row>
     <row r="19">
@@ -1295,7 +1469,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_standard</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1304,19 +1478,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.87</v>
+        <v>0.906740902763969</v>
       </c>
       <c r="E19" t="n">
-        <v>0.036</v>
+        <v>0.0142634886677039</v>
       </c>
       <c r="F19" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.1166523366580106</v>
       </c>
       <c r="G19" t="n">
-        <v>0.052</v>
+        <v>0.0705727554903101</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2</v>
+        <v>0.2405357765743042</v>
       </c>
     </row>
     <row r="20">
@@ -1327,28 +1501,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.852</v>
+        <v>0.822875816993464</v>
       </c>
       <c r="E20" t="n">
-        <v>0.12</v>
+        <v>0.0414032201524907</v>
       </c>
       <c r="F20" t="n">
-        <v>0.228</v>
+        <v>0.1459121874376871</v>
       </c>
       <c r="G20" t="n">
-        <v>0.16</v>
+        <v>0.1277821366654725</v>
       </c>
       <c r="H20" t="n">
-        <v>0.6200000000000001</v>
+        <v>0.4029759316695724</v>
       </c>
     </row>
     <row r="21">
@@ -1359,28 +1533,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>dirichlet</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.852</v>
+        <v>0.8235294117647058</v>
       </c>
       <c r="E21" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0317551010811806</v>
       </c>
       <c r="F21" t="n">
-        <v>0.1026</v>
+        <v>0.088359769420743</v>
       </c>
       <c r="G21" t="n">
-        <v>0.07200000000000002</v>
+        <v>0.1260980249403627</v>
       </c>
       <c r="H21" t="n">
-        <v>0.2790000000000001</v>
+        <v>0.3965582009347524</v>
       </c>
     </row>
     <row r="22">
@@ -1396,23 +1570,23 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.852</v>
+        <v>0.8846782097353806</v>
       </c>
       <c r="E22" t="n">
-        <v>0.04800000000000001</v>
+        <v>0.018769244883138</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0912</v>
+        <v>0.1825360274188585</v>
       </c>
       <c r="G22" t="n">
-        <v>0.06400000000000002</v>
+        <v>0.08647635999389899</v>
       </c>
       <c r="H22" t="n">
-        <v>0.2480000000000001</v>
+        <v>0.2866155484462337</v>
       </c>
     </row>
     <row r="23">
@@ -1423,28 +1597,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>test_dialect_barishal</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>dirichlet</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.8869650441032343</v>
       </c>
       <c r="E23" t="n">
-        <v>0.15</v>
+        <v>0.0425479165641032</v>
       </c>
       <c r="F23" t="n">
-        <v>0.276</v>
+        <v>0.1277637772827475</v>
       </c>
       <c r="G23" t="n">
-        <v>0.19</v>
+        <v>0.0882980328322521</v>
       </c>
       <c r="H23" t="n">
-        <v>0.74</v>
+        <v>0.2947132589821578</v>
       </c>
     </row>
     <row r="24">
@@ -1464,19 +1638,19 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.8908853315909834</v>
       </c>
       <c r="E24" t="n">
-        <v>0.06750000000000002</v>
+        <v>0.0263579986997657</v>
       </c>
       <c r="F24" t="n">
-        <v>0.1242</v>
+        <v>0.185892333712094</v>
       </c>
       <c r="G24" t="n">
-        <v>0.08550000000000001</v>
+        <v>0.081397387816749</v>
       </c>
       <c r="H24" t="n">
-        <v>0.333</v>
+        <v>0.2727508381473471</v>
       </c>
     </row>
     <row r="25">
@@ -1496,19 +1670,19 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.8925187847108788</v>
       </c>
       <c r="E25" t="n">
-        <v>0.06000000000000001</v>
+        <v>0.0262560687242077</v>
       </c>
       <c r="F25" t="n">
-        <v>0.1104</v>
+        <v>0.1632757809747144</v>
       </c>
       <c r="G25" t="n">
-        <v>0.07600000000000001</v>
+        <v>0.0800617410120998</v>
       </c>
       <c r="H25" t="n">
-        <v>0.296</v>
+        <v>0.2706417929268392</v>
       </c>
     </row>
     <row r="26">
@@ -1528,19 +1702,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.9</v>
+        <v>0.9013720421554982</v>
       </c>
       <c r="E26" t="n">
-        <v>0.04</v>
+        <v>0.03735281196329354</v>
       </c>
       <c r="F26" t="n">
-        <v>0.1</v>
+        <v>0.1754933487285267</v>
       </c>
       <c r="G26" t="n">
-        <v>0.08</v>
+        <v>0.07488338962241778</v>
       </c>
       <c r="H26" t="n">
-        <v>0.3</v>
+        <v>0.2558713288995172</v>
       </c>
     </row>
     <row r="27">
@@ -1560,19 +1734,19 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.9</v>
+        <v>0.9013720421554982</v>
       </c>
       <c r="E27" t="n">
-        <v>0.018</v>
+        <v>0.02274078515029186</v>
       </c>
       <c r="F27" t="n">
-        <v>0.04500000000000001</v>
+        <v>0.1624897899049701</v>
       </c>
       <c r="G27" t="n">
-        <v>0.036</v>
+        <v>0.07318905545215726</v>
       </c>
       <c r="H27" t="n">
-        <v>0.135</v>
+        <v>0.2455444377024153</v>
       </c>
     </row>
     <row r="28">
@@ -1583,28 +1757,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>test_standard</t>
+          <t>test_dialect_chittagong</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.9</v>
+        <v>0.822280300555374</v>
       </c>
       <c r="E28" t="n">
-        <v>0.016</v>
+        <v>0.08147581483790277</v>
       </c>
       <c r="F28" t="n">
-        <v>0.04000000000000001</v>
+        <v>0.1935544586181641</v>
       </c>
       <c r="G28" t="n">
-        <v>0.032</v>
+        <v>0.135771370926235</v>
       </c>
       <c r="H28" t="n">
-        <v>0.12</v>
+        <v>0.4529112768822393</v>
       </c>
     </row>
     <row r="29">
@@ -1620,23 +1794,23 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pre_calibration</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.861</v>
+        <v>0.822280300555374</v>
       </c>
       <c r="E29" t="n">
-        <v>0.105</v>
+        <v>0.05570710541200341</v>
       </c>
       <c r="F29" t="n">
-        <v>0.204</v>
+        <v>0.1172945402877432</v>
       </c>
       <c r="G29" t="n">
-        <v>0.145</v>
+        <v>0.1314018789948027</v>
       </c>
       <c r="H29" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.4203099198481008</v>
       </c>
     </row>
     <row r="30">
@@ -1647,28 +1821,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>temp_scaling</t>
+          <t>pre_calibration</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.861</v>
+        <v>0.8784710878797779</v>
       </c>
       <c r="E30" t="n">
-        <v>0.04725000000000001</v>
+        <v>0.05754346100626254</v>
       </c>
       <c r="F30" t="n">
-        <v>0.09180000000000001</v>
+        <v>0.2988440773703835</v>
       </c>
       <c r="G30" t="n">
-        <v>0.06525000000000002</v>
+        <v>0.09244130022433357</v>
       </c>
       <c r="H30" t="n">
-        <v>0.2520000000000001</v>
+        <v>0.3118115968673298</v>
       </c>
     </row>
     <row r="31">
@@ -1679,28 +1853,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>test_dialect_chittagong</t>
+          <t>test_dialect_noakhali</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>dirichlet</t>
+          <t>temp_scaling</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.861</v>
+        <v>0.8784710878797779</v>
       </c>
       <c r="E31" t="n">
-        <v>0.04200000000000001</v>
+        <v>0.04341262383024432</v>
       </c>
       <c r="F31" t="n">
-        <v>0.08160000000000001</v>
+        <v>0.2506340782936305</v>
       </c>
       <c r="G31" t="n">
-        <v>0.05800000000000001</v>
+        <v>0.09001458427702165</v>
       </c>
       <c r="H31" t="n">
-        <v>0.224</v>
+        <v>0.2953692939527402</v>
       </c>
     </row>
     <row r="32">
@@ -1711,7 +1885,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1720,19 +1894,19 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.8376</v>
+        <v>0.8895785690950669</v>
       </c>
       <c r="E32" t="n">
-        <v>0.144</v>
+        <v>0.04849258660101805</v>
       </c>
       <c r="F32" t="n">
-        <v>0.2664</v>
+        <v>0.1813300649325053</v>
       </c>
       <c r="G32" t="n">
-        <v>0.184</v>
+        <v>0.08715533582878769</v>
       </c>
       <c r="H32" t="n">
-        <v>0.7160000000000001</v>
+        <v>0.3047303237871973</v>
       </c>
     </row>
     <row r="33">
@@ -1743,7 +1917,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>test_dialect_noakhali</t>
+          <t>test_dialect_barishal</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1752,147 +1926,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.8376</v>
+        <v>0.8895785690950669</v>
       </c>
       <c r="E33" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.02866007203746761</v>
       </c>
       <c r="F33" t="n">
-        <v>0.11988</v>
+        <v>0.2090202941084808</v>
       </c>
       <c r="G33" t="n">
-        <v>0.08280000000000001</v>
+        <v>0.08524382535808468</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3222</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>test_dialect_noakhali</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0.8376</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0.05760000000000001</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0.10656</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0.07360000000000001</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.2864</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>pre_calibration</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0.8142</v>
-      </c>
-      <c r="E35" t="n">
-        <v>0.183</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0.3288</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0.223</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.8720000000000001</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>temp_scaling</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0.8142</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0.08235000000000001</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0.14796</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0.10035</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.3924000000000001</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>0.8142</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0.07320000000000002</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0.13152</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.08920000000000002</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.3488000000000001</v>
+        <v>0.2875104668385335</v>
       </c>
     </row>
   </sheetData>
@@ -1906,7 +1952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1948,7 +1994,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.044</v>
+        <v>0.0150269772184873</v>
       </c>
     </row>
     <row r="3">
@@ -1968,7 +2014,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.0308</v>
+        <v>0.0150269772184873</v>
       </c>
     </row>
     <row r="4">
@@ -1988,7 +2034,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.0296</v>
+        <v>0.0146842032963466</v>
       </c>
     </row>
     <row r="5">
@@ -2008,7 +2054,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.074</v>
+        <v>0.06268836436599259</v>
       </c>
     </row>
     <row r="6">
@@ -2028,7 +2074,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.0443</v>
+        <v>0.06268836436599259</v>
       </c>
     </row>
     <row r="7">
@@ -2048,7 +2094,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.0416</v>
+        <v>0.0603275096731152</v>
       </c>
     </row>
     <row r="8">
@@ -2068,7 +2114,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.09200000000000001</v>
+        <v>0.0195901163438971</v>
       </c>
     </row>
     <row r="9">
@@ -2088,7 +2134,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0524</v>
+        <v>0.0195901163438971</v>
       </c>
     </row>
     <row r="10">
@@ -2108,7 +2154,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.04880000000000001</v>
+        <v>0.0196833361420656</v>
       </c>
     </row>
     <row r="11">
@@ -2128,7 +2174,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.11</v>
+        <v>0.0191900968897351</v>
       </c>
     </row>
     <row r="12">
@@ -2148,7 +2194,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.06050000000000001</v>
+        <v>0.0191900968897351</v>
       </c>
     </row>
     <row r="13">
@@ -2168,7 +2214,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05600000000000001</v>
+        <v>0.0184023349325937</v>
       </c>
     </row>
     <row r="14">
@@ -2188,7 +2234,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.044</v>
+        <v>0.0235138588363206</v>
       </c>
     </row>
     <row r="15">
@@ -2208,7 +2254,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.0308</v>
+        <v>0.0235138588363206</v>
       </c>
     </row>
     <row r="16">
@@ -2228,7 +2274,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0296</v>
+        <v>0.0236797019800191</v>
       </c>
     </row>
     <row r="17">
@@ -2248,7 +2294,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.074</v>
+        <v>0.0705477333470443</v>
       </c>
     </row>
     <row r="18">
@@ -2268,7 +2314,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.0443</v>
+        <v>0.0705477333470443</v>
       </c>
     </row>
     <row r="19">
@@ -2288,7 +2334,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0416</v>
+        <v>0.06949519506158</v>
       </c>
     </row>
     <row r="20">
@@ -2308,7 +2354,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.09200000000000001</v>
+        <v>0.0331164636028199</v>
       </c>
     </row>
     <row r="21">
@@ -2328,7 +2374,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.0524</v>
+        <v>0.0331164636028199</v>
       </c>
     </row>
     <row r="22">
@@ -2348,7 +2394,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.04880000000000001</v>
+        <v>0.0361683048692378</v>
       </c>
     </row>
     <row r="23">
@@ -2368,7 +2414,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.11</v>
+        <v>0.0301208861315635</v>
       </c>
     </row>
     <row r="24">
@@ -2388,7 +2434,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.06050000000000001</v>
+        <v>0.0301208861315635</v>
       </c>
     </row>
     <row r="25">
@@ -2408,247 +2454,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.05600000000000001</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>test_standard</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>pre_calibration</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>0.044</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>test_standard</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>temp_scaling</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>0.0308</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>test_standard</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>0.0296</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>test_dialect_chittagong</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>pre_calibration</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>0.083</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>test_dialect_chittagong</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>temp_scaling</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>0.04835</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>test_dialect_chittagong</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>0.0452</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>test_dialect_noakhali</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>pre_calibration</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>0.1064</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>test_dialect_noakhali</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>temp_scaling</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>0.05888</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>test_dialect_noakhali</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>0.05456000000000001</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>pre_calibration</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>0.1298</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>temp_scaling</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>0.06941</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>0.06392</v>
+        <v>0.0310058578010288</v>
       </c>
     </row>
   </sheetData>
@@ -2662,7 +2468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2700,17 +2506,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>chittagong</t>
+          <t>barishal</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.62</v>
+        <v>0.2988288242213471</v>
       </c>
       <c r="D2" t="n">
-        <v>0.03000000000000003</v>
+        <v>0.01098275542526339</v>
       </c>
       <c r="E2" t="n">
-        <v>0.05</v>
+        <v>0.009889093718103099</v>
       </c>
     </row>
     <row r="3">
@@ -2725,13 +2531,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.51</v>
+        <v>0.2688565697091273</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04800000000000004</v>
+        <v>0.01882333040076156</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08000000000000002</v>
+        <v>0.007482272263382397</v>
       </c>
     </row>
     <row r="4">
@@ -2742,44 +2548,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>barishal</t>
+          <t>chittagong</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.4</v>
+        <v>0.1451302048316973</v>
       </c>
       <c r="D4" t="n">
-        <v>0.06599999999999995</v>
+        <v>0.08486640231753872</v>
       </c>
       <c r="E4" t="n">
-        <v>0.11</v>
+        <v>0.05617020149743429</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>distilbert_multi</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>chittagong</t>
+          <t>barishal</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.62</v>
+        <v>0.2988288242213471</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03900000000000003</v>
+        <v>0.01486133772697262</v>
       </c>
       <c r="E5" t="n">
-        <v>0.065</v>
+        <v>0.002893616368964298</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>distilbert_multi</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2788,97 +2594,34 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.51</v>
+        <v>0.2688565697091273</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06240000000000001</v>
+        <v>0.02106845958257542</v>
       </c>
       <c r="E6" t="n">
-        <v>0.104</v>
+        <v>-0.008465664190199298</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>distilbert_multi</t>
+          <t>xlmr_base</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>barishal</t>
+          <t>chittagong</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.4</v>
+        <v>0.1451302048316973</v>
       </c>
       <c r="D7" t="n">
-        <v>0.08579999999999999</v>
+        <v>0.08287085232449198</v>
       </c>
       <c r="E7" t="n">
-        <v>0.143</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>xlmr_base</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>chittagong</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.03000000000000003</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>xlmr_base</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>noakhali</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.04800000000000004</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.08000000000000002</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>xlmr_base</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>barishal</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.06599999999999995</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.11</v>
+        <v>0.0230455987044549</v>
       </c>
     </row>
   </sheetData>
@@ -2929,10 +2672,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9</v>
+        <v>0.9270232650626368</v>
       </c>
       <c r="D2" t="n">
-        <v>0.04</v>
+        <v>0.0357962132354742</v>
       </c>
     </row>
     <row r="3">
@@ -2947,10 +2690,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.87</v>
+        <v>0.842156862745098</v>
       </c>
       <c r="D3" t="n">
-        <v>0.09</v>
+        <v>0.09196641473290849</v>
       </c>
     </row>
     <row r="4">
@@ -2965,10 +2708,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.852</v>
+        <v>0.9081999346618752</v>
       </c>
       <c r="D4" t="n">
-        <v>0.12</v>
+        <v>0.0432784854988566</v>
       </c>
     </row>
     <row r="5">
@@ -2983,10 +2726,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.9160405096373734</v>
       </c>
       <c r="D5" t="n">
-        <v>0.15</v>
+        <v>0.0456853069535773</v>
       </c>
     </row>
     <row r="6">
@@ -3001,10 +2744,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9</v>
+        <v>0.905746669317956</v>
       </c>
       <c r="D6" t="n">
-        <v>0.04</v>
+        <v>0.0293490971321137</v>
       </c>
     </row>
     <row r="7">
@@ -3019,10 +2762,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.87</v>
+        <v>0.822875816993464</v>
       </c>
       <c r="D7" t="n">
-        <v>0.09</v>
+        <v>0.0523946958365686</v>
       </c>
     </row>
     <row r="8">
@@ -3037,10 +2780,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.852</v>
+        <v>0.8846782097353806</v>
       </c>
       <c r="D8" t="n">
-        <v>0.12</v>
+        <v>0.0208834329419144</v>
       </c>
     </row>
     <row r="9">
@@ -3055,10 +2798,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8340000000000001</v>
+        <v>0.8908853315909834</v>
       </c>
       <c r="D9" t="n">
-        <v>0.15</v>
+        <v>0.032242713501078</v>
       </c>
     </row>
     <row r="10">
@@ -3073,10 +2816,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9</v>
+        <v>0.9013720421554982</v>
       </c>
       <c r="D10" t="n">
-        <v>0.04</v>
+        <v>0.03735281196329354</v>
       </c>
     </row>
     <row r="11">
@@ -3091,10 +2834,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.861</v>
+        <v>0.822280300555374</v>
       </c>
       <c r="D11" t="n">
-        <v>0.105</v>
+        <v>0.08147581483790277</v>
       </c>
     </row>
     <row r="12">
@@ -3109,10 +2852,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.8376</v>
+        <v>0.8784710878797779</v>
       </c>
       <c r="D12" t="n">
-        <v>0.144</v>
+        <v>0.05754346100626254</v>
       </c>
     </row>
     <row r="13">
@@ -3127,10 +2870,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.8142</v>
+        <v>0.8895785690950669</v>
       </c>
       <c r="D13" t="n">
-        <v>0.183</v>
+        <v>0.04849258660101805</v>
       </c>
     </row>
   </sheetData>
@@ -3144,7 +2887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3196,13 +2939,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.022</v>
+        <v>0.017176771125692</v>
       </c>
       <c r="E2" t="n">
-        <v>0.04</v>
+        <v>0.0357962132354742</v>
       </c>
       <c r="F2" t="n">
-        <v>0.018</v>
+        <v>0.0186194421097822</v>
       </c>
     </row>
     <row r="3">
@@ -3222,13 +2965,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.0495</v>
+        <v>0.02326000228957699</v>
       </c>
       <c r="E3" t="n">
-        <v>0.09</v>
+        <v>0.09196641473290849</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0405</v>
+        <v>0.0687064124433315</v>
       </c>
     </row>
     <row r="4">
@@ -3248,13 +2991,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.066</v>
+        <v>0.0193591030605885</v>
       </c>
       <c r="E4" t="n">
-        <v>0.12</v>
+        <v>0.0432784854988566</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.0239193824382681</v>
       </c>
     </row>
     <row r="5">
@@ -3274,13 +3017,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0825</v>
+        <v>0.0140160774749164</v>
       </c>
       <c r="E5" t="n">
-        <v>0.15</v>
+        <v>0.0456853069535773</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06750000000000002</v>
+        <v>0.0316692294786609</v>
       </c>
     </row>
     <row r="6">
@@ -3300,13 +3043,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.024</v>
+        <v>0.0225072705641798</v>
       </c>
       <c r="E6" t="n">
-        <v>0.04</v>
+        <v>0.0357962132354742</v>
       </c>
       <c r="F6" t="n">
-        <v>0.016</v>
+        <v>0.0132889426712944</v>
       </c>
     </row>
     <row r="7">
@@ -3326,13 +3069,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.054</v>
+        <v>0.0383915478283036</v>
       </c>
       <c r="E7" t="n">
-        <v>0.09</v>
+        <v>0.09196641473290849</v>
       </c>
       <c r="F7" t="n">
-        <v>0.036</v>
+        <v>0.0535748669046049</v>
       </c>
     </row>
     <row r="8">
@@ -3352,13 +3095,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.020072753454881</v>
       </c>
       <c r="E8" t="n">
-        <v>0.12</v>
+        <v>0.0432784854988566</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04800000000000001</v>
+        <v>0.0232057320439756</v>
       </c>
     </row>
     <row r="9">
@@ -3378,13 +3121,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.09000000000000001</v>
+        <v>0.0228286074200879</v>
       </c>
       <c r="E9" t="n">
-        <v>0.15</v>
+        <v>0.0456853069535773</v>
       </c>
       <c r="F9" t="n">
-        <v>0.06000000000000001</v>
+        <v>0.0228566995334894</v>
       </c>
     </row>
     <row r="10">
@@ -3404,13 +3147,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.022</v>
+        <v>0.003838971775897801</v>
       </c>
       <c r="E10" t="n">
-        <v>0.04</v>
+        <v>0.0293490971321137</v>
       </c>
       <c r="F10" t="n">
-        <v>0.018</v>
+        <v>0.0255101253562159</v>
       </c>
     </row>
     <row r="11">
@@ -3430,13 +3173,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.0495</v>
+        <v>0.0109914756840779</v>
       </c>
       <c r="E11" t="n">
-        <v>0.09</v>
+        <v>0.0523946958365686</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0405</v>
+        <v>0.0414032201524907</v>
       </c>
     </row>
     <row r="12">
@@ -3456,13 +3199,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.066</v>
+        <v>0.0021141880587764</v>
       </c>
       <c r="E12" t="n">
-        <v>0.12</v>
+        <v>0.0208834329419144</v>
       </c>
       <c r="F12" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.018769244883138</v>
       </c>
     </row>
     <row r="13">
@@ -3482,13 +3225,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.0825</v>
+        <v>0.005884714801312297</v>
       </c>
       <c r="E13" t="n">
-        <v>0.15</v>
+        <v>0.032242713501078</v>
       </c>
       <c r="F13" t="n">
-        <v>0.06750000000000002</v>
+        <v>0.0263579986997657</v>
       </c>
     </row>
     <row r="14">
@@ -3508,13 +3251,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.024</v>
+        <v>0.0150856084644098</v>
       </c>
       <c r="E14" t="n">
-        <v>0.04</v>
+        <v>0.0293490971321137</v>
       </c>
       <c r="F14" t="n">
-        <v>0.016</v>
+        <v>0.0142634886677039</v>
       </c>
     </row>
     <row r="15">
@@ -3534,13 +3277,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.054</v>
+        <v>0.020639594755388</v>
       </c>
       <c r="E15" t="n">
-        <v>0.09</v>
+        <v>0.0523946958365686</v>
       </c>
       <c r="F15" t="n">
-        <v>0.036</v>
+        <v>0.0317551010811806</v>
       </c>
     </row>
     <row r="16">
@@ -3560,13 +3303,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.07200000000000001</v>
+        <v>-0.0216644836221888</v>
       </c>
       <c r="E16" t="n">
-        <v>0.12</v>
+        <v>0.0208834329419144</v>
       </c>
       <c r="F16" t="n">
-        <v>0.04800000000000001</v>
+        <v>0.0425479165641032</v>
       </c>
     </row>
     <row r="17">
@@ -3586,13 +3329,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.09000000000000001</v>
+        <v>0.005986644776870297</v>
       </c>
       <c r="E17" t="n">
-        <v>0.15</v>
+        <v>0.032242713501078</v>
       </c>
       <c r="F17" t="n">
-        <v>0.06000000000000001</v>
+        <v>0.0262560687242077</v>
       </c>
     </row>
     <row r="18">
@@ -3612,13 +3355,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.022</v>
+        <v>0.01461202681300168</v>
       </c>
       <c r="E18" t="n">
-        <v>0.04</v>
+        <v>0.03735281196329354</v>
       </c>
       <c r="F18" t="n">
-        <v>0.018</v>
+        <v>0.02274078515029186</v>
       </c>
     </row>
     <row r="19">
@@ -3638,13 +3381,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.05775</v>
+        <v>0.02576870942589936</v>
       </c>
       <c r="E19" t="n">
-        <v>0.105</v>
+        <v>0.08147581483790277</v>
       </c>
       <c r="F19" t="n">
-        <v>0.04725000000000001</v>
+        <v>0.05570710541200341</v>
       </c>
     </row>
     <row r="20">
@@ -3664,13 +3407,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.01413083717601823</v>
       </c>
       <c r="E20" t="n">
-        <v>0.144</v>
+        <v>0.05754346100626254</v>
       </c>
       <c r="F20" t="n">
-        <v>0.06480000000000001</v>
+        <v>0.04341262383024432</v>
       </c>
     </row>
     <row r="21">
@@ -3690,117 +3433,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.10065</v>
+        <v>0.01983251456355044</v>
       </c>
       <c r="E21" t="n">
-        <v>0.183</v>
+        <v>0.04849258660101805</v>
       </c>
       <c r="F21" t="n">
-        <v>0.08235000000000001</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>test_standard</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.016</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>test_dialect_chittagong</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="E23" t="n">
-        <v>0.105</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.04200000000000001</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>test_dialect_noakhali</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0.0864</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.05760000000000001</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>distilbert_multi</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>test_dialect_barishal</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>dirichlet</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>0.1098</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.183</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0.07320000000000002</v>
+        <v>0.02866007203746761</v>
       </c>
     </row>
   </sheetData>
@@ -3842,17 +3481,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>chittagong</t>
+          <t>barishal</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.62</v>
+        <v>0.2988288242213471</v>
       </c>
       <c r="C2" t="n">
-        <v>3200</v>
+        <v>10034</v>
       </c>
       <c r="D2" t="n">
-        <v>1984</v>
+        <v>5843</v>
       </c>
     </row>
     <row r="3">
@@ -3862,29 +3501,29 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.51</v>
+        <v>0.2688565697091273</v>
       </c>
       <c r="C3" t="n">
-        <v>3100</v>
+        <v>9939</v>
       </c>
       <c r="D3" t="n">
-        <v>1581</v>
+        <v>5361</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>barishal</t>
+          <t>chittagong</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4</v>
+        <v>0.1451302048316973</v>
       </c>
       <c r="C4" t="n">
-        <v>3050</v>
+        <v>10187</v>
       </c>
       <c r="D4" t="n">
-        <v>1220</v>
+        <v>3238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>